<commit_message>
Tool and criteria: seed the defuel scenarios through DefuelService
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WhWgyuDz8T5X2xkvgDd6W
</commit_message>
<xml_diff>
--- a/docs/test-data/scenarios/JetBlue_B6_Scenario_Seed_2026-09-24_to_26.xlsx
+++ b/docs/test-data/scenarios/JetBlue_B6_Scenario_Seed_2026-09-24_to_26.xlsx
@@ -32605,7 +32605,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>PARTIAL - the defuel and its charge are seeded</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -32650,7 +32650,7 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>Not demonstrable until movement type / DEFUEL_SERVICE charge exist. Data is ready in PROPOSED_DEFUEL_* sheets.</t>
+          <t>Defueling app: the defuel (TO_SUPPLIER, PARKED) carries the service charge in defuel_charges_usd. Matching the supplier's service invoice needs a DEFUEL_SERVICE charge type on invoice lines, which does not exist. Seeded by tools/seed-defuel-scenarios.js.</t>
         </is>
       </c>
     </row>
@@ -32665,7 +32665,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>PARTIAL - the defuel and its charge are seeded</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -32710,7 +32710,7 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>Not demonstrable until movement type / DEFUEL_SERVICE charge exist. Data is ready in PROPOSED_DEFUEL_* sheets.</t>
+          <t>Defueling app: the defuel (TO_SUPPLIER, PARKED) carries the service charge in defuel_charges_usd. Matching the supplier's service invoice needs a DEFUEL_SERVICE charge type on invoice lines, which does not exist. Seeded by tools/seed-defuel-scenarios.js.</t>
         </is>
       </c>
     </row>
@@ -32725,7 +32725,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>PARTIAL - the defuel and its charge are seeded</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -32770,7 +32770,7 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>Not demonstrable until movement type / DEFUEL_SERVICE charge exist. Data is ready in PROPOSED_DEFUEL_* sheets.</t>
+          <t>Defueling app: the defuel (TO_SUPPLIER, PARKED) carries the service charge in defuel_charges_usd. Matching the supplier's service invoice needs a DEFUEL_SERVICE charge type on invoice lines, which does not exist. Seeded by tools/seed-defuel-scenarios.js.</t>
         </is>
       </c>
     </row>
@@ -32785,7 +32785,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL - shows the gap</t>
+          <t>YES (B6) - expected credit; credit memo when that branch merges</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -32830,7 +32830,7 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>Load the credit note as an invoice and Validate: INV456 HARD on the negative line (no field marks a defuel). Full demo needs document_type CREDIT_NOTE.</t>
+          <t>Defueling app: the defuel is posted to the supplier (POSTING_PENDING) with its expected credit; 12C credits 300 L less and writes the rest off. ExpectedCredits on the invoice service lists them. TP is not seeded: expected credits are USD-only in the credit memo R1.</t>
         </is>
       </c>
     </row>
@@ -32845,7 +32845,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL - shows the gap</t>
+          <t>YES (B6) - expected credit; credit memo when that branch merges</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -32890,7 +32890,7 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>Load the credit note as an invoice and Validate: INV456 HARD on the negative line (no field marks a defuel). Full demo needs document_type CREDIT_NOTE.</t>
+          <t>Defueling app: the defuel is posted to the supplier (POSTING_PENDING) with its expected credit; 12C credits 300 L less and writes the rest off. ExpectedCredits on the invoice service lists them. TP is not seeded: expected credits are USD-only in the credit memo R1.</t>
         </is>
       </c>
     </row>
@@ -32905,7 +32905,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>PARTIAL - shows the gap</t>
+          <t>YES (B6) - expected credit; credit memo when that branch merges</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -32950,7 +32950,7 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>Load the credit note as an invoice and Validate: INV456 HARD on the negative line (no field marks a defuel). Full demo needs document_type CREDIT_NOTE.</t>
+          <t>Defueling app: the defuel is posted to the supplier (POSTING_PENDING) with its expected credit; 12C credits 300 L less and writes the rest off. ExpectedCredits on the invoice service lists them. TP is not seeded: expected credits are USD-only in the credit memo R1.</t>
         </is>
       </c>
     </row>
@@ -32965,7 +32965,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -33006,7 +33006,7 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>Needs storage-location master and movement type. Data ready in PROPOSED_DEFUEL_TICKETS / PROPOSED_STORAGE_LOCATIONS.</t>
+          <t>Defueling app: the defuel moves the fuel into the station's TEMP tank; the stock valuation shows the batch leaving the tail and arriving in the tank at its own rate, and ROB falls by the same amount.</t>
         </is>
       </c>
     </row>
@@ -33021,7 +33021,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -33062,7 +33062,7 @@
       </c>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>Needs storage-location master and movement type. Data ready in PROPOSED_DEFUEL_TICKETS / PROPOSED_STORAGE_LOCATIONS.</t>
+          <t>Defueling app: the defuel moves the fuel into the station's TEMP tank; the stock valuation shows the batch leaving the tail and arriving in the tank at its own rate, and ROB falls by the same amount.</t>
         </is>
       </c>
     </row>
@@ -33077,7 +33077,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>NO - needs schema (proposed sheets)</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -33118,7 +33118,7 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>Needs storage-location master and movement type. Data ready in PROPOSED_DEFUEL_TICKETS / PROPOSED_STORAGE_LOCATIONS.</t>
+          <t>Defueling app: the defuel moves the fuel into the station's TEMP tank; the stock valuation shows the batch leaving the tail and arriving in the tank at its own rate, and ROB falls by the same amount.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Workbooks: defuel figures as seeded, not as proposed
tools/seed-defuel-scenarios.js cuts a proposed defuel the tail cannot spare
(DFL432), so the two scenario workbooks still showed the proposed litres,
charges and credits. tools/scenario-seed/sync-defuel-figures.py rewrites
them from db/data/fuelsphere-DEFUEL.csv: Scenario_Index text, the
PROPOSED_DEFUEL_* sheets and the S17e/f/g expected journal entries. Credits
are valued from the tail's FIFO layers (12A 3305.92, 12B 1405.95, 12C
2309.23 with 391.84 written off), storage defuels go to the station's TEMP
tank. TAP scenario 12 is not seeded and stays as proposed. Re-running the
tool changes nothing.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011WhWgyuDz8T5X2xkvgDd6W
</commit_message>
<xml_diff>
--- a/docs/test-data/scenarios/JetBlue_B6_Scenario_Seed_2026-09-24_to_26.xlsx
+++ b/docs/test-data/scenarios/JetBlue_B6_Scenario_Seed_2026-09-24_to_26.xlsx
@@ -28255,12 +28255,12 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>16311.08</t>
+          <t>16311.06</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>-1835.17</t>
+          <t>-1835.19</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
@@ -28382,7 +28382,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>-2867.00</t>
+          <t>-1480.00</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -28402,12 +28402,12 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>7342.23</t>
+          <t>8460.58</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>-2311.66</t>
+          <t>-1193.31</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
@@ -28529,7 +28529,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>-3354.00</t>
+          <t>-3340.00</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -28549,12 +28549,12 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>6424.93</t>
+          <t>6428.96</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>-2671.80</t>
+          <t>-2667.77</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
@@ -28696,12 +28696,12 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>16458.22</t>
+          <t>16456.91</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>-2032.86</t>
+          <t>-2034.16</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
@@ -28823,7 +28823,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-2153.00</t>
+          <t>-1110.00</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -28843,12 +28843,12 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>6727.93</t>
+          <t>7562.36</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>-1720.68</t>
+          <t>-886.25</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
@@ -28990,12 +28990,12 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>18698.79</t>
+          <t>18698.78</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>-1665.98</t>
+          <t>-1665.99</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
@@ -29137,12 +29137,12 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>17825.26</t>
+          <t>17827.55</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>-1905.56</t>
+          <t>-1903.27</t>
         </is>
       </c>
       <c r="R8" t="inlineStr">
@@ -29222,7 +29222,7 @@
       </c>
       <c r="AZ8" t="inlineStr">
         <is>
-          <t>BOS-FS01</t>
+          <t>BOS-TEMP</t>
         </is>
       </c>
       <c r="BA8" t="inlineStr">
@@ -29269,7 +29269,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>-3389.00</t>
+          <t>-3060.00</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -29289,12 +29289,12 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>14783.98</t>
+          <t>15050.95</t>
         </is>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>-2738.65</t>
+          <t>-2471.68</t>
         </is>
       </c>
       <c r="R9" t="inlineStr">
@@ -29374,7 +29374,7 @@
       </c>
       <c r="AZ9" t="inlineStr">
         <is>
-          <t>BOS-FS01</t>
+          <t>BOS-TEMP</t>
         </is>
       </c>
       <c r="BA9" t="inlineStr">
@@ -29526,7 +29526,7 @@
       </c>
       <c r="AZ10" t="inlineStr">
         <is>
-          <t>LHR-FS01</t>
+          <t>LHR-TEMP</t>
         </is>
       </c>
       <c r="BA10" t="inlineStr">
@@ -31495,7 +31495,7 @@
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-WFS-HPN-26092411B (-2867 L) and a service invoice DFS-WFS-HPN-260924B: 2867 L x 0.032/L. Aircraft change after fuelling (tail swap); fuel taken off the original tail by the supplier.</t>
+          <t>Defuel ticket DF-WFS-HPN-26092411B (-1480 L) and a service invoice DFS-WFS-HPN-260924B: 1480 L x 0.032/L. Aircraft change after fuelling (tail swap); fuel taken off the original tail by the supplier. [Seeded at 1480 L, cut from the proposed 2867 L: the tail could not spare more (DFL432).]</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -31555,7 +31555,7 @@
       </c>
       <c r="J34" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-WFS-BNA-26092511C (-3354 L) and a service invoice DFS-WFS-BNA-260925C: 3354 L x 0.032/L. Fuel quality hold - supplier defuelled for sampling, service charged.</t>
+          <t>Defuel ticket DF-WFS-BNA-26092511C (-3340 L) and a service invoice DFS-WFS-BNA-260925C: 3340 L x 0.032/L. Fuel quality hold - supplier defuelled for sampling, service charged. [Seeded at 3340 L, cut from the proposed 3354 L: the tail could not spare more (DFL432).]</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
@@ -31615,7 +31615,7 @@
       </c>
       <c r="J35" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-CGA-SFO-26092512A (-2530 L) and credit note CN-CGA-SFO-260925A for -2530 L at the uplift price. Flight cancelled after fuelling; fuel returned to the supplier, credit note expected.</t>
+          <t>Defuel ticket DF-CGA-SFO-26092512A (-2530 L) and credit note CN-CGA-SFO-260925A for -2530 L at the value drawn from the tail's FIFO layers. Flight cancelled after fuelling; fuel returned to the supplier, credit note expected.</t>
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr">
@@ -31675,7 +31675,7 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-WFS-BDL-26092512B (-2153 L) and credit note CN-WFS-BDL-260925B for -2153 L at the uplift price. Over-fuelled by the supplier against the order; excess returned for credit.</t>
+          <t>Defuel ticket DF-WFS-BDL-26092512B (-1110 L) and credit note CN-WFS-BDL-260925B for -1110 L at the value drawn from the tail's FIFO layers. Over-fuelled by the supplier against the order; excess returned for credit. [Seeded at 1110 L, cut from the proposed 2153 L: the tail could not spare more (DFL432).]</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -31735,7 +31735,7 @@
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-SHL-BOS-26092412C (-2068 L) and credit note CN-SHL-BOS-260924C for -1768 L at the uplift price. Contamination suspected; fuel returned, part credited and part disposed (write-off).</t>
+          <t>Defuel ticket DF-SHL-BOS-26092412C (-2068 L) and credit note CN-SHL-BOS-260924C for -1768 L at the value drawn from the tail's FIFO layers. Contamination suspected; fuel returned, part credited and part disposed (write-off).</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -31791,12 +31791,12 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-SHL-BOS-26092613A (-2354 L) with disposition STORAGE to BOS-FS01; no invoice. Tankering plan cancelled; fuel moved to the airline storage tank at the station.</t>
+          <t>Defuel ticket DF-SHL-BOS-26092613A (-2354 L) with disposition STORAGE to BOS-TEMP; no invoice. Tankering plan cancelled; fuel moved to the airline storage tank at the station.</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Fuel moves from the tail to storage location BOS-FS01 (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
+          <t>Fuel moves from the tail to storage location BOS-TEMP (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
         </is>
       </c>
       <c r="L38" s="2" t="inlineStr">
@@ -31847,12 +31847,12 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-WFS-BOS-26092513B (-3389 L) with disposition STORAGE to BOS-FS01; no invoice. Defuel ahead of a heavy check; fuel held in the airline storage tank for re-use.</t>
+          <t>Defuel ticket DF-WFS-BOS-26092513B (-3060 L) with disposition STORAGE to BOS-TEMP; no invoice. Defuel ahead of a heavy check; fuel held in the airline storage tank for re-use. [Seeded at 3060 L, cut from the proposed 3389 L: the tail could not spare more (DFL432).]</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Fuel moves from the tail to storage location BOS-FS01 (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
+          <t>Fuel moves from the tail to storage location BOS-TEMP (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -31903,12 +31903,12 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Defuel ticket DF-BPK-LHR-26092413C (-3828 L) with disposition STORAGE to LHR-FS01; no invoice. Fuel transferred off the tail into the airline storage tank pending re-uplift.</t>
+          <t>Defuel ticket DF-BPK-LHR-26092413C (-3828 L) with disposition STORAGE to LHR-TEMP; no invoice. Fuel transferred off the tail into the airline storage tank pending re-uplift.</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Fuel moves from the tail to storage location LHR-FS01 (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
+          <t>Fuel moves from the tail to storage location LHR-TEMP (no supplier, no invoice). The ROB ledger takes a DEFUEL/TRANSFER out of the tail; stock moves into the storage location (S/4 transfer posting). NEEDS SCHEMA: storage location master + movement type on the ticket.</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -32988,7 +32988,7 @@
       </c>
       <c r="V2" t="inlineStr">
         <is>
-          <t>-1835.17</t>
+          <t>-1835.19</t>
         </is>
       </c>
       <c r="X2" t="inlineStr">
@@ -33120,7 +33120,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>-2867.00</t>
+          <t>-1480.00</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -33150,7 +33150,7 @@
       </c>
       <c r="V3" t="inlineStr">
         <is>
-          <t>-2311.66</t>
+          <t>-1193.31</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
@@ -33282,7 +33282,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>-3354.00</t>
+          <t>-3340.00</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
@@ -33312,7 +33312,7 @@
       </c>
       <c r="V4" t="inlineStr">
         <is>
-          <t>-2671.80</t>
+          <t>-2667.77</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
@@ -33474,7 +33474,7 @@
       </c>
       <c r="V5" t="inlineStr">
         <is>
-          <t>-2032.86</t>
+          <t>-2034.16</t>
         </is>
       </c>
       <c r="X5" t="inlineStr">
@@ -33606,7 +33606,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>-2153.00</t>
+          <t>-1110.00</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
@@ -33636,7 +33636,7 @@
       </c>
       <c r="V6" t="inlineStr">
         <is>
-          <t>-1720.68</t>
+          <t>-886.25</t>
         </is>
       </c>
       <c r="X6" t="inlineStr">
@@ -33798,7 +33798,7 @@
       </c>
       <c r="V7" t="inlineStr">
         <is>
-          <t>-1665.98</t>
+          <t>-1665.99</t>
         </is>
       </c>
       <c r="X7" t="inlineStr">
@@ -33960,7 +33960,7 @@
       </c>
       <c r="V8" t="inlineStr">
         <is>
-          <t>-1905.56</t>
+          <t>-1903.27</t>
         </is>
       </c>
       <c r="X8" t="inlineStr">
@@ -34030,7 +34030,7 @@
       </c>
       <c r="AQ8" t="inlineStr">
         <is>
-          <t>BOS-FS01</t>
+          <t>BOS-TEMP</t>
         </is>
       </c>
       <c r="AR8" t="inlineStr">
@@ -34097,7 +34097,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>-3389.00</t>
+          <t>-3060.00</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
@@ -34127,7 +34127,7 @@
       </c>
       <c r="V9" t="inlineStr">
         <is>
-          <t>-2738.65</t>
+          <t>-2471.68</t>
         </is>
       </c>
       <c r="X9" t="inlineStr">
@@ -34197,7 +34197,7 @@
       </c>
       <c r="AQ9" t="inlineStr">
         <is>
-          <t>BOS-FS01</t>
+          <t>BOS-TEMP</t>
         </is>
       </c>
       <c r="AR9" t="inlineStr">
@@ -34364,7 +34364,7 @@
       </c>
       <c r="AQ10" t="inlineStr">
         <is>
-          <t>LHR-FS01</t>
+          <t>LHR-TEMP</t>
         </is>
       </c>
       <c r="AR10" t="inlineStr">
@@ -35980,7 +35980,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2867.000</t>
+          <t>1480.000</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -35995,7 +35995,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>91.74</t>
+          <t>47.36</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -36092,7 +36092,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>3354.000</t>
+          <t>3340.000</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -36107,7 +36107,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>107.33</t>
+          <t>106.88</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -36214,12 +36214,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1.3161</t>
+          <t>1.3067</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>-3329.73</t>
+          <t>-3305.92</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -36321,7 +36321,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>-2153.000</t>
+          <t>-1110.000</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -36331,12 +36331,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1.3516</t>
+          <t>1.2666</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>-2909.99</t>
+          <t>-1405.95</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -36453,7 +36453,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>-2309.18</t>
+          <t>-2309.23</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -36606,7 +36606,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BOS-FS01</t>
+          <t>BOS-TEMP</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -36648,7 +36648,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>LHR-FS01</t>
+          <t>LHR-TEMP</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -38408,7 +38408,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>3329.73</t>
+          <t>3305.92</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -38423,7 +38423,7 @@
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>2530 L x 1.3161</t>
+          <t>2530 L returned, valued from the tail's FIFO layers at 3305.92</t>
         </is>
       </c>
     </row>
@@ -38468,7 +38468,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>3329.73</t>
+          <t>3305.92</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -38483,7 +38483,7 @@
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>2530 L x 1.3161</t>
+          <t>2530 L returned, valued from the tail's FIFO layers at 3305.92</t>
         </is>
       </c>
     </row>
@@ -38528,7 +38528,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>3329.73</t>
+          <t>3305.92</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -38588,7 +38588,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>3329.73</t>
+          <t>3305.92</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -38888,7 +38888,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>2309.18</t>
+          <t>2309.23</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -38903,7 +38903,7 @@
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>2068 L defuelled, 300 L disposed, at 1.3061</t>
+          <t>2068 L defuelled worth 2701.07 (FIFO layers); 1768 L credited, 300 L disposed</t>
         </is>
       </c>
     </row>
@@ -38948,7 +38948,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>391.83</t>
+          <t>391.84</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -38963,7 +38963,7 @@
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>2068 L defuelled, 300 L disposed, at 1.3061</t>
+          <t>2068 L defuelled worth 2701.07 (FIFO layers); 1768 L credited, 300 L disposed</t>
         </is>
       </c>
     </row>
@@ -39008,7 +39008,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>2701.01</t>
+          <t>2701.07</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -39023,7 +39023,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>2068 L defuelled, 300 L disposed, at 1.3061</t>
+          <t>2068 L defuelled worth 2701.07 (FIFO layers); 1768 L credited, 300 L disposed</t>
         </is>
       </c>
     </row>

</xml_diff>